<commit_message>
Regenerate schemas, mock data, docs and workbook template
The generators had never been run against the last two dictionary changes,
so the app was reading a repCount that mock-data.js no longer carried and
knew nothing about meeting attendees.

- SourceStratum gains repCount; SourcePayDashboard loses it
- The RepsRecruited table is gone
- Meetings gains attendees, with two sample rows left blank to stand for
  rows logged before the column existed

The .xlsx changes shape here rather than just churning bytes, so it is
committed: it supersedes the previous template.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0199coiY3PAZyQmqXFCGrbDY
</commit_message>
<xml_diff>
--- a/london-mapping/workbook-template/London_Project_Mapping_template.xlsx
+++ b/london-mapping/workbook-template/London_Project_Mapping_template.xlsx
@@ -1,28 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SourceGIAS" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SourceStratum" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SourcePayDashboard" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SourceWorkforceSurvey" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WCtoURN" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MatAliases" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldNotes" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DisputeTracker" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BranchFacts" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MatFacts" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Meetings" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RepsRecruited" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RepCommittees" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Snapshots" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reconciliations" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SchoolGeo" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="SourceGIAS" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="SourceStratum" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="SourcePayDashboard" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="SourceWorkforceSurvey" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="WCtoURN" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="MatAliases" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="FieldNotes" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="DisputeTracker" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="BranchFacts" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="MatFacts" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Meetings" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="RepCommittees" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Snapshots" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Reconciliations" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="SchoolGeo" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -194,34 +193,21 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="Meetings" displayName="Meetings" ref="A1:D2" headerRowCount="1">
-  <autoFilter ref="A1:D2"/>
-  <tableColumns count="4">
-    <tableColumn id="1" name="ID"/>
-    <tableColumn id="2" name="Date"/>
-    <tableColumn id="3" name="URN"/>
-    <tableColumn id="4" name="Logged by"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
-</table>
-</file>
-
-<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="RepsRecruited" displayName="RepsRecruited" ref="A1:E2" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="Meetings" displayName="Meetings" ref="A1:E2" headerRowCount="1">
   <autoFilter ref="A1:E2"/>
   <tableColumns count="5">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Date"/>
     <tableColumn id="3" name="URN"/>
-    <tableColumn id="4" name="Rep name"/>
-    <tableColumn id="5" name="Logged by"/>
+    <tableColumn id="4" name="Logged by"/>
+    <tableColumn id="5" name="Attendees"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
 </file>
 
-<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="RepCommittees" displayName="RepCommittees" ref="A1:E2" headerRowCount="1">
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="RepCommittees" displayName="RepCommittees" ref="A1:E2" headerRowCount="1">
   <autoFilter ref="A1:E2"/>
   <tableColumns count="5">
     <tableColumn id="1" name="ID"/>
@@ -234,8 +220,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="Snapshots" displayName="Snapshots" ref="A1:K2" headerRowCount="1">
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="Snapshots" displayName="Snapshots" ref="A1:K2" headerRowCount="1">
   <autoFilter ref="A1:K2"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Snapshot date"/>
@@ -254,8 +240,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="Reconciliations" displayName="Reconciliations" ref="A1:H2" headerRowCount="1">
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="Reconciliations" displayName="Reconciliations" ref="A1:H2" headerRowCount="1">
   <autoFilter ref="A1:H2"/>
   <tableColumns count="8">
     <tableColumn id="1" name="ID"/>
@@ -271,8 +257,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="SchoolGeo" displayName="SchoolGeo" ref="A1:D2" headerRowCount="1">
+<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="SchoolGeo" displayName="SchoolGeo" ref="A1:D2" headerRowCount="1">
   <autoFilter ref="A1:D2"/>
   <tableColumns count="4">
     <tableColumn id="1" name="URN"/>
@@ -285,9 +271,9 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="SourceStratum" displayName="SourceStratum" ref="A1:K2" headerRowCount="1">
-  <autoFilter ref="A1:K2"/>
-  <tableColumns count="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="SourceStratum" displayName="SourceStratum" ref="A1:L2" headerRowCount="1">
+  <autoFilter ref="A1:L2"/>
+  <tableColumns count="12">
     <tableColumn id="1" name="Workplace code"/>
     <tableColumn id="2" name="Workplace name"/>
     <tableColumn id="3" name="Headcount (total)"/>
@@ -298,37 +284,37 @@
     <tableColumn id="8" name="Membership (teachers)"/>
     <tableColumn id="9" name="Membership (leadership)"/>
     <tableColumn id="10" name="Membership (support)"/>
-    <tableColumn id="11" name="Export date"/>
+    <tableColumn id="11" name="Rep count"/>
+    <tableColumn id="12" name="Export date"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcePayDashboard" displayName="SourcePayDashboard" ref="A1:U2" headerRowCount="1">
-  <autoFilter ref="A1:U2"/>
-  <tableColumns count="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcePayDashboard" displayName="SourcePayDashboard" ref="A1:T2" headerRowCount="1">
+  <autoFilter ref="A1:T2"/>
+  <tableColumns count="20">
     <tableColumn id="1" name="Workplace code"/>
     <tableColumn id="2" name="Workplace name"/>
-    <tableColumn id="3" name="Rep count"/>
-    <tableColumn id="4" name="Members voted (2026 indicative)"/>
-    <tableColumn id="5" name="Members voted (2025 indicative)"/>
-    <tableColumn id="6" name="Members voted (2024 indicative)"/>
-    <tableColumn id="7" name="Turnout (2026 indicative)"/>
-    <tableColumn id="8" name="Volunteers"/>
-    <tableColumn id="9" name="WP conversations"/>
-    <tableColumn id="10" name="Active SEVs"/>
-    <tableColumn id="11" name="Rep recruited volunteer"/>
-    <tableColumn id="12" name="Joined community"/>
-    <tableColumn id="13" name="Completed activate action"/>
-    <tableColumn id="14" name="Agreed to briefing"/>
-    <tableColumn id="15" name="Hold a meeting"/>
-    <tableColumn id="16" name="Needs support"/>
-    <tableColumn id="17" name="Pledged to vote"/>
-    <tableColumn id="18" name="Branch name"/>
-    <tableColumn id="19" name="District name"/>
-    <tableColumn id="20" name="Region name"/>
-    <tableColumn id="21" name="Import date"/>
+    <tableColumn id="3" name="Members voted (2026 indicative)"/>
+    <tableColumn id="4" name="Members voted (2025 indicative)"/>
+    <tableColumn id="5" name="Members voted (2024 indicative)"/>
+    <tableColumn id="6" name="Turnout (2026 indicative)"/>
+    <tableColumn id="7" name="Volunteers"/>
+    <tableColumn id="8" name="WP conversations"/>
+    <tableColumn id="9" name="Active SEVs"/>
+    <tableColumn id="10" name="Rep recruited volunteer"/>
+    <tableColumn id="11" name="Joined community"/>
+    <tableColumn id="12" name="Completed activate action"/>
+    <tableColumn id="13" name="Agreed to briefing"/>
+    <tableColumn id="14" name="Hold a meeting"/>
+    <tableColumn id="15" name="Needs support"/>
+    <tableColumn id="16" name="Pledged to vote"/>
+    <tableColumn id="17" name="Branch name"/>
+    <tableColumn id="18" name="District name"/>
+    <tableColumn id="19" name="Region name"/>
+    <tableColumn id="20" name="Import date"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -1084,85 +1070,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>URN</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Logged by</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>m1</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>2026-01-20</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>100097</v>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>EXAMPLE Organiser</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Note: Written by the app from a school's page. Branch and project meeting counts derive from this — do not keep a separate tally.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Column order must match data-dictionary/dictionary.json — the app reads columns by position.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1191,24 +1098,24 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Rep name</t>
+          <t>Logged by</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Logged by</t>
+          <t>Attendees</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>r1</t>
+          <t>m1</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
@@ -1216,19 +1123,17 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>EXAMPLE Rep</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
           <t>EXAMPLE Organiser</t>
         </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Note: Written by the app from a school's page. Distinct from reps TRAINED, which is still a manual figure on BranchFacts.</t>
+          <t>Note: Written by the app from a school's page. Branch and project meeting counts derive from this — do not keep a separate tally. Attendees is the organiser's count on the day and may be approximate; it is blank on rows logged before that column existed.</t>
         </is>
       </c>
     </row>
@@ -1247,7 +1152,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1339,7 +1244,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1477,7 +1382,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1607,7 +1512,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1688,7 +1593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1701,7 +1606,8 @@
     <col width="23" customWidth="1" min="8" max="8"/>
     <col width="25" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1757,6 +1663,11 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>Rep count</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>Export date</t>
         </is>
       </c>
@@ -1796,7 +1707,10 @@
       <c r="J2" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>2026-07-21</t>
         </is>
@@ -1805,7 +1719,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Note: Paste your Stratum export here (the 'Full Membership List for Stats purposes' report). This is the primary source for headcount and membership — the workforce survey's headcount is treated as a third-party cross-check. Not edited by the app.</t>
+          <t>Note: Paste your Stratum export here (the 'Full Membership List for Stats purposes' report). This is the primary source for headcount, membership and rep count — the workforce survey's headcount is treated as a third-party cross-check. Not edited by the app.</t>
         </is>
       </c>
     </row>
@@ -1830,30 +1744,29 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U5"/>
+  <dimension ref="A1:T5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="33" customWidth="1" min="3" max="3"/>
     <col width="33" customWidth="1" min="4" max="4"/>
     <col width="33" customWidth="1" min="5" max="5"/>
-    <col width="33" customWidth="1" min="6" max="6"/>
-    <col width="27" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="27" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
-    <col width="15" customWidth="1" min="16" max="16"/>
-    <col width="17" customWidth="1" min="17" max="17"/>
-    <col width="13" customWidth="1" min="18" max="18"/>
-    <col width="15" customWidth="1" min="19" max="19"/>
+    <col width="27" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="27" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="15" max="15"/>
+    <col width="17" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="15" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="19" max="19"/>
     <col width="13" customWidth="1" min="20" max="20"/>
-    <col width="13" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1869,95 +1782,90 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Rep count</t>
+          <t>Members voted (2026 indicative)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Members voted (2026 indicative)</t>
+          <t>Members voted (2025 indicative)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Members voted (2025 indicative)</t>
+          <t>Members voted (2024 indicative)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Members voted (2024 indicative)</t>
+          <t>Turnout (2026 indicative)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Turnout (2026 indicative)</t>
+          <t>Volunteers</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Volunteers</t>
+          <t>WP conversations</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>WP conversations</t>
+          <t>Active SEVs</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Active SEVs</t>
+          <t>Rep recruited volunteer</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Rep recruited volunteer</t>
+          <t>Joined community</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Joined community</t>
+          <t>Completed activate action</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Completed activate action</t>
+          <t>Agreed to briefing</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Agreed to briefing</t>
+          <t>Hold a meeting</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Hold a meeting</t>
+          <t>Needs support</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>Needs support</t>
+          <t>Pledged to vote</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>Pledged to vote</t>
+          <t>Branch name</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>Branch name</t>
+          <t>District name</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>District name</t>
+          <t>Region name</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>Region name</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Import date</t>
         </is>
@@ -1975,66 +1883,63 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>0.736</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="I2" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="F2" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v>0.736</v>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="I2" s="2" t="n">
-        <v>6</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="K2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="L2" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="M2" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="L2" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="M2" s="2" t="n">
-        <v>9</v>
       </c>
       <c r="N2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="O2" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="2" t="n">
         <v>5</v>
       </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>Greenwich State Education</t>
+        </is>
+      </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>Greenwich State Education</t>
+          <t>Greenwich</t>
         </is>
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
-          <t>Greenwich</t>
+          <t>London</t>
         </is>
       </c>
       <c r="T2" s="2" t="inlineStr">
-        <is>
-          <t>London</t>
-        </is>
-      </c>
-      <c r="U2" s="2" t="inlineStr">
         <is>
           <t>2026-07-21</t>
         </is>
@@ -2043,7 +1948,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Note: Paste your NEU Pay Dashboard export here. Membership and headcount now come from Stratum instead — this source covers ballots, engagement and rep count. Not edited by the app.</t>
+          <t>Note: Paste your NEU Pay Dashboard export here. Membership and headcount come from Stratum, and so does the rep count — this source covers ballots and engagement. Not edited by the app.</t>
         </is>
       </c>
     </row>

</xml_diff>